<commit_message>
solve + tight layout
</commit_message>
<xml_diff>
--- a/dambreak_experimental_data.xlsx
+++ b/dambreak_experimental_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Mines IC\TR Fluide\VS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9682BF-E5F8-478D-A0DB-6705590143DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16878D67-75AA-4A0D-B9C8-F2F18D354EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" tabRatio="902" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="902" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="experiments_Pashias_et_al_1996" sheetId="34" r:id="rId1"/>
@@ -1507,7 +1507,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1663,12 +1663,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -1712,6 +1725,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1743,16 +1771,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2078,40 +2096,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="15" thickBot="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="26"/>
-      <c r="F1" s="21" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="31"/>
+      <c r="F1" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
-      <c r="Z1" s="22"/>
-      <c r="AA1" s="22"/>
-      <c r="AB1" s="22"/>
-      <c r="AC1" s="22"/>
-      <c r="AD1" s="22"/>
-      <c r="AE1" s="23"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="27"/>
+      <c r="AA1" s="27"/>
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="28"/>
     </row>
     <row r="2" spans="1:31" ht="22" thickBot="1">
       <c r="A2" s="11" t="s">
@@ -2129,7 +2147,7 @@
       <c r="F2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="35" t="s">
+      <c r="G2" s="21" t="s">
         <v>8</v>
       </c>
       <c r="H2" s="6" t="s">
@@ -7137,40 +7155,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="15" thickBot="1">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="29"/>
-      <c r="F1" s="21" t="s">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="34"/>
+      <c r="F1" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
-      <c r="Z1" s="22"/>
-      <c r="AA1" s="22"/>
-      <c r="AB1" s="22"/>
-      <c r="AC1" s="22"/>
-      <c r="AD1" s="22"/>
-      <c r="AE1" s="23"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="27"/>
+      <c r="AA1" s="27"/>
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="28"/>
     </row>
     <row r="2" spans="1:31" ht="22" thickBot="1">
       <c r="A2" s="9" t="s">
@@ -18934,39 +18952,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="15" thickBot="1">
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="30"/>
-      <c r="D1" s="31"/>
-      <c r="F1" s="21" t="s">
+      <c r="C1" s="35"/>
+      <c r="D1" s="36"/>
+      <c r="F1" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
-      <c r="Z1" s="22"/>
-      <c r="AA1" s="22"/>
-      <c r="AB1" s="22"/>
-      <c r="AC1" s="22"/>
-      <c r="AD1" s="22"/>
-      <c r="AE1" s="23"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="27"/>
+      <c r="AA1" s="27"/>
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="28"/>
     </row>
     <row r="2" spans="1:31" ht="22" thickBot="1">
       <c r="A2" t="s">
@@ -21917,40 +21935,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="15" thickBot="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="26"/>
-      <c r="F1" s="21" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="31"/>
+      <c r="F1" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
-      <c r="Z1" s="22"/>
-      <c r="AA1" s="22"/>
-      <c r="AB1" s="22"/>
-      <c r="AC1" s="22"/>
-      <c r="AD1" s="22"/>
-      <c r="AE1" s="23"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="27"/>
+      <c r="AA1" s="27"/>
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="28"/>
     </row>
     <row r="2" spans="1:31" ht="22" thickBot="1">
       <c r="A2" s="11" t="s">
@@ -26714,41 +26732,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="15" thickBot="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="32"/>
-      <c r="G1" s="21" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="24"/>
+      <c r="G1" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
-      <c r="Z1" s="22"/>
-      <c r="AA1" s="22"/>
-      <c r="AB1" s="22"/>
-      <c r="AC1" s="22"/>
-      <c r="AD1" s="22"/>
-      <c r="AE1" s="22"/>
-      <c r="AF1" s="23"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="27"/>
+      <c r="AA1" s="27"/>
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="27"/>
+      <c r="AF1" s="28"/>
     </row>
     <row r="2" spans="1:32" ht="22" thickBot="1">
       <c r="A2" s="11" t="s">
@@ -26760,10 +26778,10 @@
       <c r="C2" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="32" t="s">
+      <c r="E2" s="25" t="s">
         <v>57</v>
       </c>
       <c r="G2" s="6" t="s">
@@ -26855,10 +26873,10 @@
       <c r="C3" s="17">
         <v>4.9366800944725796E-3</v>
       </c>
-      <c r="D3" s="17">
+      <c r="D3" s="22">
         <v>0.11</v>
       </c>
-      <c r="E3" s="33">
+      <c r="E3" s="17">
         <f>1-C3/I3</f>
         <v>0.94910639077863324</v>
       </c>
@@ -26972,10 +26990,10 @@
       <c r="C4" s="16">
         <v>1.3051800308956699E-2</v>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="23">
         <v>0.09</v>
       </c>
-      <c r="E4" s="33">
+      <c r="E4" s="16">
         <f t="shared" ref="E4:E10" si="11">1-C4/I4</f>
         <v>0.86544535763962172</v>
       </c>
@@ -27089,10 +27107,10 @@
       <c r="C5" s="16">
         <v>1.4134501705755099E-2</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="23">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="E5" s="33">
+      <c r="E5" s="16">
         <f t="shared" si="11"/>
         <v>0.85428348756953509</v>
       </c>
@@ -27206,10 +27224,10 @@
       <c r="C6" s="16">
         <v>1.8323409021429399E-2</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="23">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E6" s="33">
+      <c r="E6" s="16">
         <f t="shared" si="11"/>
         <v>0.81109887606773823</v>
       </c>
@@ -27323,10 +27341,10 @@
       <c r="C7" s="16">
         <v>2.4006373924264999E-2</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="23">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="E7" s="33">
+      <c r="E7" s="16">
         <f t="shared" si="11"/>
         <v>0.75251160902819592</v>
       </c>
@@ -27440,10 +27458,10 @@
       <c r="C8" s="16">
         <v>2.6979338854154499E-2</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="23">
         <v>0.05</v>
       </c>
-      <c r="E8" s="33">
+      <c r="E8" s="16">
         <f t="shared" si="11"/>
         <v>0.72186248603964431</v>
       </c>
@@ -27557,10 +27575,10 @@
       <c r="C9" s="16">
         <v>5.1033598372430801E-2</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="23">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="E9" s="33">
+      <c r="E9" s="16">
         <f t="shared" si="11"/>
         <v>0.4738804291501979</v>
       </c>
@@ -27674,10 +27692,10 @@
       <c r="C10" s="16">
         <v>9.7000000000000003E-2</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="23">
         <v>3.2000000000000001E-2</v>
       </c>
-      <c r="E10" s="33">
+      <c r="E10" s="16">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -27920,42 +27938,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="15" thickBot="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="26"/>
-      <c r="H1" s="21" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="31"/>
+      <c r="H1" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
-      <c r="Z1" s="22"/>
-      <c r="AA1" s="22"/>
-      <c r="AB1" s="22"/>
-      <c r="AC1" s="22"/>
-      <c r="AD1" s="22"/>
-      <c r="AE1" s="22"/>
-      <c r="AF1" s="22"/>
-      <c r="AG1" s="23"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="27"/>
+      <c r="AA1" s="27"/>
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="27"/>
+      <c r="AF1" s="27"/>
+      <c r="AG1" s="28"/>
     </row>
     <row r="2" spans="1:33" ht="22" thickBot="1">
       <c r="A2" s="11" t="s">
@@ -32139,47 +32157,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="15" thickBot="1">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="32"/>
-      <c r="M1" s="21" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="24"/>
+      <c r="M1" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="22"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
-      <c r="T1" s="22"/>
-      <c r="U1" s="22"/>
-      <c r="V1" s="22"/>
-      <c r="W1" s="22"/>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
-      <c r="Z1" s="22"/>
-      <c r="AA1" s="22"/>
-      <c r="AB1" s="22"/>
-      <c r="AC1" s="22"/>
-      <c r="AD1" s="22"/>
-      <c r="AE1" s="22"/>
-      <c r="AF1" s="22"/>
-      <c r="AG1" s="22"/>
-      <c r="AH1" s="22"/>
-      <c r="AI1" s="22"/>
-      <c r="AJ1" s="22"/>
-      <c r="AK1" s="22"/>
-      <c r="AL1" s="23"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27"/>
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="27"/>
+      <c r="AA1" s="27"/>
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="27"/>
+      <c r="AF1" s="27"/>
+      <c r="AG1" s="27"/>
+      <c r="AH1" s="27"/>
+      <c r="AI1" s="27"/>
+      <c r="AJ1" s="27"/>
+      <c r="AK1" s="27"/>
+      <c r="AL1" s="28"/>
     </row>
     <row r="2" spans="1:38" ht="30.5" thickBot="1">
       <c r="A2" s="15" t="s">
@@ -32212,7 +32230,7 @@
       <c r="J2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="K2" s="32" t="s">
+      <c r="K2" s="25" t="s">
         <v>57</v>
       </c>
       <c r="M2" s="6" t="s">
@@ -32329,7 +32347,7 @@
         <f t="shared" ref="J3:J44" si="1">G3*D3</f>
         <v>0.23346829394620042</v>
       </c>
-      <c r="K3" s="34">
+      <c r="K3" s="2">
         <f>1-I3</f>
         <v>0.13408222253304114</v>
       </c>
@@ -32468,7 +32486,7 @@
         <f t="shared" si="1"/>
         <v>0.1306456933828542</v>
       </c>
-      <c r="K4" s="34">
+      <c r="K4" s="1">
         <f t="shared" ref="K4:K44" si="16">1-I4</f>
         <v>0.29581005645683067</v>
       </c>
@@ -32607,7 +32625,7 @@
         <f t="shared" si="1"/>
         <v>0.22973101875887003</v>
       </c>
-      <c r="K5" s="34">
+      <c r="K5" s="1">
         <f t="shared" si="16"/>
         <v>0.14568619461707311</v>
       </c>
@@ -32746,7 +32764,7 @@
         <f t="shared" si="1"/>
         <v>3.5967907442691363E-2</v>
       </c>
-      <c r="K6" s="34">
+      <c r="K6" s="1">
         <f t="shared" si="16"/>
         <v>0.67258149255054911</v>
       </c>
@@ -32885,7 +32903,7 @@
         <f t="shared" si="1"/>
         <v>3.9006426718167453E-2</v>
       </c>
-      <c r="K7" s="34">
+      <c r="K7" s="1">
         <f t="shared" si="16"/>
         <v>0.65847320100499673</v>
       </c>
@@ -33024,7 +33042,7 @@
         <f t="shared" si="1"/>
         <v>4.4548014950936007E-2</v>
       </c>
-      <c r="K8" s="34">
+      <c r="K8" s="1">
         <f t="shared" si="16"/>
         <v>0.67989810724215616</v>
       </c>
@@ -33163,7 +33181,7 @@
         <f t="shared" si="1"/>
         <v>4.6568856061430478E-2</v>
       </c>
-      <c r="K9" s="34">
+      <c r="K9" s="1">
         <f t="shared" si="16"/>
         <v>0.64514418745701918</v>
       </c>
@@ -33302,7 +33320,7 @@
         <f t="shared" si="1"/>
         <v>8.7667893586354934E-2</v>
       </c>
-      <c r="K10" s="34">
+      <c r="K10" s="1">
         <f t="shared" si="16"/>
         <v>0.44107669986741693</v>
       </c>
@@ -33441,7 +33459,7 @@
         <f t="shared" si="1"/>
         <v>8.8676701339438807E-2</v>
       </c>
-      <c r="K11" s="34">
+      <c r="K11" s="1">
         <f t="shared" si="16"/>
         <v>0.52259089137258752</v>
       </c>
@@ -33580,7 +33598,7 @@
         <f t="shared" si="1"/>
         <v>9.0703993658585808E-2</v>
       </c>
-      <c r="K12" s="34">
+      <c r="K12" s="1">
         <f t="shared" si="16"/>
         <v>0.52259089137258752</v>
       </c>
@@ -33719,7 +33737,7 @@
         <f t="shared" si="1"/>
         <v>9.7293096896355707E-2</v>
       </c>
-      <c r="K13" s="34">
+      <c r="K13" s="1">
         <f t="shared" si="16"/>
         <v>0.44942474445650893</v>
       </c>
@@ -33858,7 +33876,7 @@
         <f t="shared" si="1"/>
         <v>9.8301098248358129E-2</v>
       </c>
-      <c r="K14" s="34">
+      <c r="K14" s="1">
         <f t="shared" si="16"/>
         <v>0.43968013697787423</v>
       </c>
@@ -33997,7 +34015,7 @@
         <f t="shared" si="1"/>
         <v>8.8651702905908861E-2</v>
       </c>
-      <c r="K15" s="34">
+      <c r="K15" s="1">
         <f t="shared" si="16"/>
         <v>0.52614369313453824</v>
       </c>
@@ -34136,7 +34154,7 @@
         <f t="shared" si="1"/>
         <v>0.1191231805764018</v>
       </c>
-      <c r="K16" s="34">
+      <c r="K16" s="1">
         <f t="shared" si="16"/>
         <v>0.38174605855913668</v>
       </c>
@@ -34275,7 +34293,7 @@
         <f t="shared" si="1"/>
         <v>0.12317534601145146</v>
       </c>
-      <c r="K17" s="34">
+      <c r="K17" s="1">
         <f t="shared" si="16"/>
         <v>0.42381659303588137</v>
       </c>
@@ -34414,7 +34432,7 @@
         <f t="shared" si="1"/>
         <v>0.12570663900659967</v>
       </c>
-      <c r="K18" s="34">
+      <c r="K18" s="1">
         <f t="shared" si="16"/>
         <v>0.3700394750525634</v>
       </c>
@@ -34553,7 +34571,7 @@
         <f t="shared" si="1"/>
         <v>0.15313556539620826</v>
       </c>
-      <c r="K19" s="34">
+      <c r="K19" s="1">
         <f t="shared" si="16"/>
         <v>0.35430875346560919</v>
       </c>
@@ -34692,7 +34710,7 @@
         <f t="shared" si="1"/>
         <v>0.15464676102313044</v>
       </c>
-      <c r="K20" s="34">
+      <c r="K20" s="1">
         <f t="shared" si="16"/>
         <v>0.3709433235149423</v>
       </c>
@@ -34831,7 +34849,7 @@
         <f t="shared" si="1"/>
         <v>0.18969295202955069</v>
       </c>
-      <c r="K21" s="34">
+      <c r="K21" s="1">
         <f t="shared" si="16"/>
         <v>0.30675075797015683</v>
       </c>
@@ -34970,7 +34988,7 @@
         <f t="shared" si="1"/>
         <v>0.24695579944632695</v>
       </c>
-      <c r="K22" s="34">
+      <c r="K22" s="1">
         <f t="shared" si="16"/>
         <v>0.14817590662752689</v>
       </c>
@@ -35109,7 +35127,7 @@
         <f t="shared" si="1"/>
         <v>0.1643823740223864</v>
       </c>
-      <c r="K23" s="34">
+      <c r="K23" s="1">
         <f t="shared" si="16"/>
         <v>0.28081419538366548</v>
       </c>
@@ -35248,7 +35266,7 @@
         <f t="shared" si="1"/>
         <v>0.10392803204433837</v>
       </c>
-      <c r="K24" s="34">
+      <c r="K24" s="1">
         <f t="shared" si="16"/>
         <v>0.40196296060671355</v>
       </c>
@@ -35387,7 +35405,7 @@
         <f t="shared" si="1"/>
         <v>0.12473106808357136</v>
       </c>
-      <c r="K25" s="34">
+      <c r="K25" s="1">
         <f t="shared" si="16"/>
         <v>0.34691352601820979</v>
       </c>
@@ -35526,7 +35544,7 @@
         <f t="shared" si="1"/>
         <v>0.14901436009166155</v>
       </c>
-      <c r="K26" s="34">
+      <c r="K26" s="1">
         <f t="shared" si="16"/>
         <v>0.40363771831092432</v>
       </c>
@@ -35665,7 +35683,7 @@
         <f t="shared" si="1"/>
         <v>0.1973492300933356</v>
       </c>
-      <c r="K27" s="34">
+      <c r="K27" s="1">
         <f t="shared" si="16"/>
         <v>0.3727173943296731</v>
       </c>
@@ -35804,7 +35822,7 @@
         <f t="shared" si="1"/>
         <v>0.20940090804052375</v>
       </c>
-      <c r="K28" s="34">
+      <c r="K28" s="1">
         <f t="shared" si="16"/>
         <v>0.21462536282398248</v>
       </c>
@@ -35943,7 +35961,7 @@
         <f t="shared" si="1"/>
         <v>0.26161290322580599</v>
       </c>
-      <c r="K29" s="34">
+      <c r="K29" s="1">
         <f t="shared" si="16"/>
         <v>0.15505226480836298</v>
       </c>
@@ -36082,7 +36100,7 @@
         <f t="shared" si="1"/>
         <v>0.176199436763952</v>
       </c>
-      <c r="K30" s="34">
+      <c r="K30" s="1">
         <f t="shared" si="16"/>
         <v>0.25958188153310102</v>
       </c>
@@ -36221,7 +36239,7 @@
         <f t="shared" si="1"/>
         <v>7.7177419354838697E-2</v>
       </c>
-      <c r="K31" s="34">
+      <c r="K31" s="1">
         <f t="shared" si="16"/>
         <v>0.45999999999999996</v>
       </c>
@@ -36360,7 +36378,7 @@
         <f t="shared" si="1"/>
         <v>8.2037890424987103E-2</v>
       </c>
-      <c r="K32" s="34">
+      <c r="K32" s="1">
         <f t="shared" si="16"/>
         <v>0.44999999999999996</v>
       </c>
@@ -36499,7 +36517,7 @@
         <f t="shared" si="1"/>
         <v>0.12328085606040508</v>
       </c>
-      <c r="K33" s="34">
+      <c r="K33" s="1">
         <f t="shared" si="16"/>
         <v>0.3448146514477759</v>
       </c>
@@ -36638,7 +36656,7 @@
         <f t="shared" si="1"/>
         <v>0.15814859246684407</v>
       </c>
-      <c r="K34" s="34">
+      <c r="K34" s="1">
         <f t="shared" si="16"/>
         <v>0.28930022790198917</v>
       </c>
@@ -36777,7 +36795,7 @@
         <f t="shared" si="1"/>
         <v>2.2987038402957318E-2</v>
       </c>
-      <c r="K35" s="34">
+      <c r="K35" s="1">
         <f t="shared" si="16"/>
         <v>0.77645484604977466</v>
       </c>
@@ -36916,7 +36934,7 @@
         <f t="shared" si="1"/>
         <v>3.128320026281798E-2</v>
       </c>
-      <c r="K36" s="34">
+      <c r="K36" s="1">
         <f t="shared" si="16"/>
         <v>0.73036306173014043</v>
       </c>
@@ -37055,7 +37073,7 @@
         <f t="shared" si="1"/>
         <v>3.9552946078547084E-2</v>
       </c>
-      <c r="K37" s="34">
+      <c r="K37" s="1">
         <f t="shared" si="16"/>
         <v>0.73497224016210372</v>
       </c>
@@ -37194,7 +37212,7 @@
         <f t="shared" si="1"/>
         <v>4.7233918910651235E-2</v>
       </c>
-      <c r="K38" s="34">
+      <c r="K38" s="1">
         <f t="shared" si="16"/>
         <v>0.67966209897854302</v>
       </c>
@@ -37333,7 +37351,7 @@
         <f t="shared" si="1"/>
         <v>5.4277350677656759E-2</v>
       </c>
-      <c r="K39" s="34">
+      <c r="K39" s="1">
         <f t="shared" si="16"/>
         <v>0.6439409661308263</v>
       </c>
@@ -37472,7 +37490,7 @@
         <f t="shared" si="1"/>
         <v>6.4828528304826105E-2</v>
       </c>
-      <c r="K40" s="34">
+      <c r="K40" s="1">
         <f t="shared" si="16"/>
         <v>0.61513360093105529</v>
       </c>
@@ -37611,7 +37629,7 @@
         <f t="shared" si="1"/>
         <v>7.6655804063890429E-2</v>
       </c>
-      <c r="K41" s="34">
+      <c r="K41" s="1">
         <f t="shared" si="16"/>
         <v>0.57365099504338724</v>
       </c>
@@ -37750,7 +37768,7 @@
         <f t="shared" si="1"/>
         <v>9.5841472116144522E-2</v>
       </c>
-      <c r="K42" s="34">
+      <c r="K42" s="1">
         <f t="shared" si="16"/>
         <v>0.55424191059680994</v>
       </c>
@@ -37889,7 +37907,7 @@
         <f t="shared" si="1"/>
         <v>0.10989785559923435</v>
       </c>
-      <c r="K43" s="34">
+      <c r="K43" s="1">
         <f t="shared" si="16"/>
         <v>0.51027479160388789</v>
       </c>
@@ -38028,7 +38046,7 @@
         <f t="shared" si="1"/>
         <v>0.10990191960602384</v>
       </c>
-      <c r="K44" s="34">
+      <c r="K44" s="1">
         <f t="shared" si="16"/>
         <v>0.51027479160388789</v>
       </c>

</xml_diff>